<commit_message>
feat: capture filament color for purchases
</commit_message>
<xml_diff>
--- a/downloads/3DTR_Quan_Ly_Kinh_Doanh_Thong_Minh.xlsx
+++ b/downloads/3DTR_Quan_Ly_Kinh_Doanh_Thong_Minh.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Mua vào" sheetId="1" r:id="R114e51f35a68461e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Tính giá" sheetId="2" r:id="Re9417bfaa166449b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Nhựa" sheetId="3" r:id="Rc32b1662929046a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Phí sàn" sheetId="4" r:id="Re90b863d1ebd42db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Danh mục" sheetId="5" r:id="R055475492d5c4281"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_Hướng dẫn" sheetId="6" r:id="Rb6d951c2aa314103"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_Đơn hàng" sheetId="7" r:id="R96b4a023f1474eb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8_Rút tiền" sheetId="8" r:id="R597b2f98f14d4f86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_Sản phẩm" sheetId="9" r:id="Rcbbc70b339c644e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Kho nhựa" sheetId="10" r:id="Rbfbf55164b694795"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Khách hàng" sheetId="11" r:id="Rc90224989bbc4178"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Đầu tư" sheetId="12" r:id="R820523a845434f2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Tài khoản" sheetId="13" r:id="Rc8c8d7b94d1d4a23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Dashboard" sheetId="14" r:id="R4105b16d5c2a4385"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Hãng nhựa" sheetId="15" r:id="R09df792edc9f4873"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Mua vào" sheetId="1" r:id="Rf43d98a360e64cfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Tính giá" sheetId="2" r:id="R8d7d194187a94f93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Nhựa" sheetId="3" r:id="R2410c41127304460"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Phí sàn" sheetId="4" r:id="Rf844b9e2f9ae4634"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Danh mục" sheetId="5" r:id="R080d44bdae47428a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_Hướng dẫn" sheetId="6" r:id="Re853ed82ef5049cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_Đơn hàng" sheetId="7" r:id="Re5dbf65f276646a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8_Rút tiền" sheetId="8" r:id="Rccb799e66e8047f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_Sản phẩm" sheetId="9" r:id="R7278acb912704c98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Kho nhựa" sheetId="10" r:id="R6e514dbd6f064a48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Khách hàng" sheetId="11" r:id="R5f530d6b7e5e469d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Đầu tư" sheetId="12" r:id="R6e1e08762fdf4184"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Tài khoản" sheetId="13" r:id="Rc3a5c69f805c43e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Dashboard" sheetId="14" r:id="Rc65141067b464004"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Hãng nhựa" sheetId="15" r:id="R33e65acf683e473a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -145,7 +145,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -220,6 +220,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFEFF6FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B1220"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -350,7 +360,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="31"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="623">
+  <x:cellXfs count="628">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
@@ -1706,6 +1716,21 @@
     <x:xf numFmtId="0" fontId="16" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1799,7 +1824,7 @@
         <x:color rgb="FFDC2626"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -1810,7 +1835,7 @@
         <x:color rgb="FF059669"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFECFDF5"/>
         </x:patternFill>
       </x:fill>
@@ -1821,7 +1846,7 @@
         <x:color rgb="FFDC2626"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -2214,7 +2239,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re8bda4228e414eac"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R86f0d56255454a6f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2244,7 +2269,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra2e8822d92ba49d2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R61ecc5e512764280"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2606,6 +2631,7 @@
     <x:col min="13" max="13" width="22" style="14" customWidth="1"/>
     <x:col min="14" max="14" width="18" style="14" customWidth="1"/>
     <x:col min="15" max="15" width="10" style="14" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="14" customFormat="1" ht="28" customHeight="1">
@@ -2634,10 +2660,8 @@
       <x:c r="O1" s="524" t="n"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="526" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Nhập dữ liệu mua vào. Khi chọn “Phụ kiện khác”, Cột C - Tên sản phẩm/phụ kiện là bắt buộc; cột K sẽ cảnh báo nếu bỏ trống.</x:t>
-        </x:is>
+      <x:c r="A2" s="526" t="str">
+        <x:v>Nhập dữ liệu mua vào. Khi chọn “Phụ kiện khác”, Cột C - Tên sản phẩm/phụ kiện là bắt buộc; khi chọn “Nhựa in”, nhập màu tại cột L để kiểm soát tồn kho theo màu.</x:v>
       </x:c>
       <x:c r="B2" s="524" t="n"/>
       <x:c r="C2" s="524" t="n"/>
@@ -2741,7 +2765,9 @@
           <x:t xml:space="preserve">Kiểm tra</x:t>
         </x:is>
       </x:c>
-      <x:c r="L4" s="524"/>
+      <x:c r="L4" s="626" t="str">
+        <x:v>Màu nhựa</x:v>
+      </x:c>
       <x:c r="M4" s="524" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Số dòng cảnh báo</x:t>
@@ -2769,7 +2795,7 @@
       <x:c r="K5" s="561" t="str">
         <x:f>IF(B5="","",IF(AND(B5="Phụ kiện khác",C5=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C5="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L5" s="524"/>
+      <x:c r="L5" s="627"/>
       <x:c r="M5" s="524" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Ngày kiểm tra</x:t>
@@ -2796,7 +2822,7 @@
       <x:c r="K6" s="561" t="str">
         <x:f>IF(B6="","",IF(AND(B6="Phụ kiện khác",C6=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C6="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L6" s="524"/>
+      <x:c r="L6" s="627"/>
       <x:c r="M6" s="524"/>
       <x:c r="N6" s="524"/>
       <x:c r="O6" s="524"/>
@@ -2817,7 +2843,7 @@
       <x:c r="K7" s="561" t="str">
         <x:f>IF(B7="","",IF(AND(B7="Phụ kiện khác",C7=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C7="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L7" s="524"/>
+      <x:c r="L7" s="627"/>
       <x:c r="M7" s="524"/>
       <x:c r="N7" s="524"/>
       <x:c r="O7" s="524"/>
@@ -2838,7 +2864,7 @@
       <x:c r="K8" s="561" t="str">
         <x:f>IF(B8="","",IF(AND(B8="Phụ kiện khác",C8=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C8="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L8" s="524"/>
+      <x:c r="L8" s="627"/>
       <x:c r="M8" s="524"/>
       <x:c r="N8" s="524"/>
       <x:c r="O8" s="524"/>
@@ -2859,7 +2885,7 @@
       <x:c r="K9" s="561" t="str">
         <x:f>IF(B9="","",IF(AND(B9="Phụ kiện khác",C9=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C9="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L9" s="524"/>
+      <x:c r="L9" s="627"/>
       <x:c r="M9" s="524"/>
       <x:c r="N9" s="524"/>
       <x:c r="O9" s="524"/>
@@ -2880,7 +2906,7 @@
       <x:c r="K10" s="561" t="str">
         <x:f>IF(B10="","",IF(AND(B10="Phụ kiện khác",C10=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C10="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L10" s="524"/>
+      <x:c r="L10" s="627"/>
       <x:c r="M10" s="524"/>
       <x:c r="N10" s="524"/>
       <x:c r="O10" s="524"/>
@@ -2901,7 +2927,7 @@
       <x:c r="K11" s="561" t="str">
         <x:f>IF(B11="","",IF(AND(B11="Phụ kiện khác",C11=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C11="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L11" s="524"/>
+      <x:c r="L11" s="627"/>
       <x:c r="M11" s="524"/>
       <x:c r="N11" s="524"/>
       <x:c r="O11" s="524"/>
@@ -2922,7 +2948,7 @@
       <x:c r="K12" s="561" t="str">
         <x:f>IF(B12="","",IF(AND(B12="Phụ kiện khác",C12=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C12="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L12" s="524"/>
+      <x:c r="L12" s="627"/>
       <x:c r="M12" s="524"/>
       <x:c r="N12" s="524"/>
       <x:c r="O12" s="524"/>
@@ -2943,7 +2969,7 @@
       <x:c r="K13" s="561" t="str">
         <x:f>IF(B13="","",IF(AND(B13="Phụ kiện khác",C13=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C13="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L13" s="524"/>
+      <x:c r="L13" s="627"/>
       <x:c r="M13" s="524"/>
       <x:c r="N13" s="524"/>
       <x:c r="O13" s="524"/>
@@ -2964,7 +2990,7 @@
       <x:c r="K14" s="561" t="str">
         <x:f>IF(B14="","",IF(AND(B14="Phụ kiện khác",C14=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C14="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L14" s="524"/>
+      <x:c r="L14" s="627"/>
       <x:c r="M14" s="524"/>
       <x:c r="N14" s="524"/>
       <x:c r="O14" s="524"/>
@@ -2985,7 +3011,7 @@
       <x:c r="K15" s="561" t="str">
         <x:f>IF(B15="","",IF(AND(B15="Phụ kiện khác",C15=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C15="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L15" s="524"/>
+      <x:c r="L15" s="627"/>
       <x:c r="M15" s="524"/>
       <x:c r="N15" s="524"/>
       <x:c r="O15" s="524"/>
@@ -3006,7 +3032,7 @@
       <x:c r="K16" s="561" t="str">
         <x:f>IF(B16="","",IF(AND(B16="Phụ kiện khác",C16=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C16="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L16" s="524"/>
+      <x:c r="L16" s="627"/>
       <x:c r="M16" s="524"/>
       <x:c r="N16" s="524"/>
       <x:c r="O16" s="524"/>
@@ -3027,7 +3053,7 @@
       <x:c r="K17" s="561" t="str">
         <x:f>IF(B17="","",IF(AND(B17="Phụ kiện khác",C17=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C17="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L17" s="524"/>
+      <x:c r="L17" s="627"/>
       <x:c r="M17" s="524"/>
       <x:c r="N17" s="524"/>
       <x:c r="O17" s="524"/>
@@ -3048,7 +3074,7 @@
       <x:c r="K18" s="561" t="str">
         <x:f>IF(B18="","",IF(AND(B18="Phụ kiện khác",C18=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C18="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L18" s="524"/>
+      <x:c r="L18" s="627"/>
       <x:c r="M18" s="524"/>
       <x:c r="N18" s="524"/>
       <x:c r="O18" s="524"/>
@@ -3069,7 +3095,7 @@
       <x:c r="K19" s="561" t="str">
         <x:f>IF(B19="","",IF(AND(B19="Phụ kiện khác",C19=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C19="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L19" s="524"/>
+      <x:c r="L19" s="627"/>
       <x:c r="M19" s="524"/>
       <x:c r="N19" s="524"/>
       <x:c r="O19" s="524"/>
@@ -3090,7 +3116,7 @@
       <x:c r="K20" s="561" t="str">
         <x:f>IF(B20="","",IF(AND(B20="Phụ kiện khác",C20=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C20="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L20" s="524"/>
+      <x:c r="L20" s="627"/>
       <x:c r="M20" s="524"/>
       <x:c r="N20" s="524"/>
       <x:c r="O20" s="524"/>
@@ -3111,7 +3137,7 @@
       <x:c r="K21" s="561" t="str">
         <x:f>IF(B21="","",IF(AND(B21="Phụ kiện khác",C21=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C21="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L21" s="524"/>
+      <x:c r="L21" s="627"/>
       <x:c r="M21" s="524"/>
       <x:c r="N21" s="524"/>
       <x:c r="O21" s="524"/>
@@ -3132,7 +3158,7 @@
       <x:c r="K22" s="561" t="str">
         <x:f>IF(B22="","",IF(AND(B22="Phụ kiện khác",C22=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C22="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L22" s="524"/>
+      <x:c r="L22" s="627"/>
       <x:c r="M22" s="524"/>
       <x:c r="N22" s="524"/>
       <x:c r="O22" s="524"/>
@@ -3153,7 +3179,7 @@
       <x:c r="K23" s="561" t="str">
         <x:f>IF(B23="","",IF(AND(B23="Phụ kiện khác",C23=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C23="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L23" s="524"/>
+      <x:c r="L23" s="627"/>
       <x:c r="M23" s="524"/>
       <x:c r="N23" s="524"/>
       <x:c r="O23" s="524"/>
@@ -3174,7 +3200,7 @@
       <x:c r="K24" s="561" t="str">
         <x:f>IF(B24="","",IF(AND(B24="Phụ kiện khác",C24=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C24="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L24" s="524"/>
+      <x:c r="L24" s="627"/>
       <x:c r="M24" s="524"/>
       <x:c r="N24" s="524"/>
       <x:c r="O24" s="524"/>
@@ -3195,7 +3221,7 @@
       <x:c r="K25" s="561" t="str">
         <x:f>IF(B25="","",IF(AND(B25="Phụ kiện khác",C25=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C25="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L25" s="524"/>
+      <x:c r="L25" s="627"/>
       <x:c r="M25" s="524"/>
       <x:c r="N25" s="524"/>
       <x:c r="O25" s="524"/>
@@ -3216,7 +3242,7 @@
       <x:c r="K26" s="561" t="str">
         <x:f>IF(B26="","",IF(AND(B26="Phụ kiện khác",C26=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C26="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L26" s="524"/>
+      <x:c r="L26" s="627"/>
       <x:c r="M26" s="524"/>
       <x:c r="N26" s="524"/>
       <x:c r="O26" s="524"/>
@@ -3237,7 +3263,7 @@
       <x:c r="K27" s="561" t="str">
         <x:f>IF(B27="","",IF(AND(B27="Phụ kiện khác",C27=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C27="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L27" s="524"/>
+      <x:c r="L27" s="627"/>
       <x:c r="M27" s="524"/>
       <x:c r="N27" s="524"/>
       <x:c r="O27" s="524"/>
@@ -3258,7 +3284,7 @@
       <x:c r="K28" s="561" t="str">
         <x:f>IF(B28="","",IF(AND(B28="Phụ kiện khác",C28=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C28="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L28" s="524"/>
+      <x:c r="L28" s="627"/>
       <x:c r="M28" s="524"/>
       <x:c r="N28" s="524"/>
       <x:c r="O28" s="524"/>
@@ -3279,7 +3305,7 @@
       <x:c r="K29" s="561" t="str">
         <x:f>IF(B29="","",IF(AND(B29="Phụ kiện khác",C29=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C29="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L29" s="524"/>
+      <x:c r="L29" s="627"/>
       <x:c r="M29" s="524"/>
       <x:c r="N29" s="524"/>
       <x:c r="O29" s="524"/>
@@ -3300,7 +3326,7 @@
       <x:c r="K30" s="561" t="str">
         <x:f>IF(B30="","",IF(AND(B30="Phụ kiện khác",C30=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C30="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L30" s="524"/>
+      <x:c r="L30" s="627"/>
       <x:c r="M30" s="524"/>
       <x:c r="N30" s="524"/>
       <x:c r="O30" s="524"/>
@@ -3321,7 +3347,7 @@
       <x:c r="K31" s="561" t="str">
         <x:f>IF(B31="","",IF(AND(B31="Phụ kiện khác",C31=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C31="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L31" s="524"/>
+      <x:c r="L31" s="627"/>
       <x:c r="M31" s="524"/>
       <x:c r="N31" s="524"/>
       <x:c r="O31" s="524"/>
@@ -3342,7 +3368,7 @@
       <x:c r="K32" s="561" t="str">
         <x:f>IF(B32="","",IF(AND(B32="Phụ kiện khác",C32=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C32="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L32" s="524"/>
+      <x:c r="L32" s="627"/>
       <x:c r="M32" s="524"/>
       <x:c r="N32" s="524"/>
       <x:c r="O32" s="524"/>
@@ -3363,7 +3389,7 @@
       <x:c r="K33" s="561" t="str">
         <x:f>IF(B33="","",IF(AND(B33="Phụ kiện khác",C33=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C33="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L33" s="524"/>
+      <x:c r="L33" s="627"/>
       <x:c r="M33" s="524"/>
       <x:c r="N33" s="524"/>
       <x:c r="O33" s="524"/>
@@ -3384,7 +3410,7 @@
       <x:c r="K34" s="561" t="str">
         <x:f>IF(B34="","",IF(AND(B34="Phụ kiện khác",C34=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C34="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L34" s="524"/>
+      <x:c r="L34" s="627"/>
       <x:c r="M34" s="524"/>
       <x:c r="N34" s="524"/>
       <x:c r="O34" s="524"/>
@@ -3405,7 +3431,7 @@
       <x:c r="K35" s="561" t="str">
         <x:f>IF(B35="","",IF(AND(B35="Phụ kiện khác",C35=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C35="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L35" s="524"/>
+      <x:c r="L35" s="627"/>
       <x:c r="M35" s="524"/>
       <x:c r="N35" s="524"/>
       <x:c r="O35" s="524"/>
@@ -3426,7 +3452,7 @@
       <x:c r="K36" s="561" t="str">
         <x:f>IF(B36="","",IF(AND(B36="Phụ kiện khác",C36=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C36="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L36" s="524"/>
+      <x:c r="L36" s="627"/>
       <x:c r="M36" s="524"/>
       <x:c r="N36" s="524"/>
       <x:c r="O36" s="524"/>
@@ -3447,7 +3473,7 @@
       <x:c r="K37" s="561" t="str">
         <x:f>IF(B37="","",IF(AND(B37="Phụ kiện khác",C37=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C37="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L37" s="524"/>
+      <x:c r="L37" s="627"/>
       <x:c r="M37" s="524"/>
       <x:c r="N37" s="524"/>
       <x:c r="O37" s="524"/>
@@ -3468,7 +3494,7 @@
       <x:c r="K38" s="561" t="str">
         <x:f>IF(B38="","",IF(AND(B38="Phụ kiện khác",C38=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C38="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L38" s="524"/>
+      <x:c r="L38" s="627"/>
       <x:c r="M38" s="524"/>
       <x:c r="N38" s="524"/>
       <x:c r="O38" s="524"/>
@@ -3489,7 +3515,7 @@
       <x:c r="K39" s="561" t="str">
         <x:f>IF(B39="","",IF(AND(B39="Phụ kiện khác",C39=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C39="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L39" s="524"/>
+      <x:c r="L39" s="627"/>
       <x:c r="M39" s="524"/>
       <x:c r="N39" s="524"/>
       <x:c r="O39" s="524"/>
@@ -3510,7 +3536,7 @@
       <x:c r="K40" s="561" t="str">
         <x:f>IF(B40="","",IF(AND(B40="Phụ kiện khác",C40=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C40="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L40" s="524"/>
+      <x:c r="L40" s="627"/>
       <x:c r="M40" s="524"/>
       <x:c r="N40" s="524"/>
       <x:c r="O40" s="524"/>
@@ -3531,7 +3557,7 @@
       <x:c r="K41" s="561" t="str">
         <x:f>IF(B41="","",IF(AND(B41="Phụ kiện khác",C41=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C41="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L41" s="524"/>
+      <x:c r="L41" s="627"/>
       <x:c r="M41" s="524"/>
       <x:c r="N41" s="524"/>
       <x:c r="O41" s="524"/>
@@ -3552,7 +3578,7 @@
       <x:c r="K42" s="561" t="str">
         <x:f>IF(B42="","",IF(AND(B42="Phụ kiện khác",C42=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C42="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L42" s="524"/>
+      <x:c r="L42" s="627"/>
       <x:c r="M42" s="524"/>
       <x:c r="N42" s="524"/>
       <x:c r="O42" s="524"/>
@@ -3573,7 +3599,7 @@
       <x:c r="K43" s="561" t="str">
         <x:f>IF(B43="","",IF(AND(B43="Phụ kiện khác",C43=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C43="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L43" s="524"/>
+      <x:c r="L43" s="627"/>
       <x:c r="M43" s="524"/>
       <x:c r="N43" s="524"/>
       <x:c r="O43" s="524"/>
@@ -3594,7 +3620,7 @@
       <x:c r="K44" s="561" t="str">
         <x:f>IF(B44="","",IF(AND(B44="Phụ kiện khác",C44=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C44="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L44" s="524"/>
+      <x:c r="L44" s="627"/>
       <x:c r="M44" s="524"/>
       <x:c r="N44" s="524"/>
       <x:c r="O44" s="524"/>
@@ -3615,7 +3641,7 @@
       <x:c r="K45" s="561" t="str">
         <x:f>IF(B45="","",IF(AND(B45="Phụ kiện khác",C45=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C45="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L45" s="524"/>
+      <x:c r="L45" s="627"/>
       <x:c r="M45" s="524"/>
       <x:c r="N45" s="524"/>
       <x:c r="O45" s="524"/>
@@ -3636,7 +3662,7 @@
       <x:c r="K46" s="561" t="str">
         <x:f>IF(B46="","",IF(AND(B46="Phụ kiện khác",C46=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C46="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L46" s="524"/>
+      <x:c r="L46" s="627"/>
       <x:c r="M46" s="524"/>
       <x:c r="N46" s="524"/>
       <x:c r="O46" s="524"/>
@@ -3657,7 +3683,7 @@
       <x:c r="K47" s="561" t="str">
         <x:f>IF(B47="","",IF(AND(B47="Phụ kiện khác",C47=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C47="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L47" s="524"/>
+      <x:c r="L47" s="627"/>
       <x:c r="M47" s="524"/>
       <x:c r="N47" s="524"/>
       <x:c r="O47" s="524"/>
@@ -3678,7 +3704,7 @@
       <x:c r="K48" s="561" t="str">
         <x:f>IF(B48="","",IF(AND(B48="Phụ kiện khác",C48=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C48="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L48" s="524"/>
+      <x:c r="L48" s="627"/>
       <x:c r="M48" s="524"/>
       <x:c r="N48" s="524"/>
       <x:c r="O48" s="524"/>
@@ -3699,7 +3725,7 @@
       <x:c r="K49" s="561" t="str">
         <x:f>IF(B49="","",IF(AND(B49="Phụ kiện khác",C49=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C49="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L49" s="524"/>
+      <x:c r="L49" s="627"/>
       <x:c r="M49" s="524"/>
       <x:c r="N49" s="524"/>
       <x:c r="O49" s="524"/>
@@ -3720,7 +3746,7 @@
       <x:c r="K50" s="561" t="str">
         <x:f>IF(B50="","",IF(AND(B50="Phụ kiện khác",C50=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C50="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L50" s="524"/>
+      <x:c r="L50" s="627"/>
       <x:c r="M50" s="524"/>
       <x:c r="N50" s="524"/>
       <x:c r="O50" s="524"/>
@@ -3741,7 +3767,7 @@
       <x:c r="K51" s="561" t="str">
         <x:f>IF(B51="","",IF(AND(B51="Phụ kiện khác",C51=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C51="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L51" s="524"/>
+      <x:c r="L51" s="627"/>
       <x:c r="M51" s="524"/>
       <x:c r="N51" s="524"/>
       <x:c r="O51" s="524"/>
@@ -3762,7 +3788,7 @@
       <x:c r="K52" s="561" t="str">
         <x:f>IF(B52="","",IF(AND(B52="Phụ kiện khác",C52=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C52="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L52" s="524"/>
+      <x:c r="L52" s="627"/>
       <x:c r="M52" s="524"/>
       <x:c r="N52" s="524"/>
       <x:c r="O52" s="524"/>
@@ -3783,7 +3809,7 @@
       <x:c r="K53" s="561" t="str">
         <x:f>IF(B53="","",IF(AND(B53="Phụ kiện khác",C53=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C53="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L53" s="524"/>
+      <x:c r="L53" s="627"/>
       <x:c r="M53" s="524"/>
       <x:c r="N53" s="524"/>
       <x:c r="O53" s="524"/>
@@ -3804,7 +3830,7 @@
       <x:c r="K54" s="561" t="str">
         <x:f>IF(B54="","",IF(AND(B54="Phụ kiện khác",C54=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C54="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L54" s="524"/>
+      <x:c r="L54" s="627"/>
       <x:c r="M54" s="524"/>
       <x:c r="N54" s="524"/>
       <x:c r="O54" s="524"/>
@@ -3825,7 +3851,7 @@
       <x:c r="K55" s="561" t="str">
         <x:f>IF(B55="","",IF(AND(B55="Phụ kiện khác",C55=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C55="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L55" s="524"/>
+      <x:c r="L55" s="627"/>
       <x:c r="M55" s="524"/>
       <x:c r="N55" s="524"/>
       <x:c r="O55" s="524"/>
@@ -3846,7 +3872,7 @@
       <x:c r="K56" s="561" t="str">
         <x:f>IF(B56="","",IF(AND(B56="Phụ kiện khác",C56=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C56="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L56" s="524"/>
+      <x:c r="L56" s="627"/>
       <x:c r="M56" s="524"/>
       <x:c r="N56" s="524"/>
       <x:c r="O56" s="524"/>
@@ -3867,7 +3893,7 @@
       <x:c r="K57" s="561" t="str">
         <x:f>IF(B57="","",IF(AND(B57="Phụ kiện khác",C57=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C57="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L57" s="524"/>
+      <x:c r="L57" s="627"/>
       <x:c r="M57" s="524"/>
       <x:c r="N57" s="524"/>
       <x:c r="O57" s="524"/>
@@ -3888,7 +3914,7 @@
       <x:c r="K58" s="561" t="str">
         <x:f>IF(B58="","",IF(AND(B58="Phụ kiện khác",C58=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C58="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L58" s="524"/>
+      <x:c r="L58" s="627"/>
       <x:c r="M58" s="524"/>
       <x:c r="N58" s="524"/>
       <x:c r="O58" s="524"/>
@@ -3909,7 +3935,7 @@
       <x:c r="K59" s="561" t="str">
         <x:f>IF(B59="","",IF(AND(B59="Phụ kiện khác",C59=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C59="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L59" s="524"/>
+      <x:c r="L59" s="627"/>
       <x:c r="M59" s="524"/>
       <x:c r="N59" s="524"/>
       <x:c r="O59" s="524"/>
@@ -3930,7 +3956,7 @@
       <x:c r="K60" s="561" t="str">
         <x:f>IF(B60="","",IF(AND(B60="Phụ kiện khác",C60=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C60="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L60" s="524"/>
+      <x:c r="L60" s="627"/>
       <x:c r="M60" s="524"/>
       <x:c r="N60" s="524"/>
       <x:c r="O60" s="524"/>
@@ -3951,7 +3977,7 @@
       <x:c r="K61" s="561" t="str">
         <x:f>IF(B61="","",IF(AND(B61="Phụ kiện khác",C61=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C61="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L61" s="524"/>
+      <x:c r="L61" s="627"/>
       <x:c r="M61" s="524"/>
       <x:c r="N61" s="524"/>
       <x:c r="O61" s="524"/>
@@ -3972,7 +3998,7 @@
       <x:c r="K62" s="561" t="str">
         <x:f>IF(B62="","",IF(AND(B62="Phụ kiện khác",C62=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C62="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L62" s="524"/>
+      <x:c r="L62" s="627"/>
       <x:c r="M62" s="524"/>
       <x:c r="N62" s="524"/>
       <x:c r="O62" s="524"/>
@@ -3993,7 +4019,7 @@
       <x:c r="K63" s="561" t="str">
         <x:f>IF(B63="","",IF(AND(B63="Phụ kiện khác",C63=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C63="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L63" s="524"/>
+      <x:c r="L63" s="627"/>
       <x:c r="M63" s="524"/>
       <x:c r="N63" s="524"/>
       <x:c r="O63" s="524"/>
@@ -4014,7 +4040,7 @@
       <x:c r="K64" s="561" t="str">
         <x:f>IF(B64="","",IF(AND(B64="Phụ kiện khác",C64=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C64="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L64" s="524"/>
+      <x:c r="L64" s="627"/>
       <x:c r="M64" s="524"/>
       <x:c r="N64" s="524"/>
       <x:c r="O64" s="524"/>
@@ -4035,7 +4061,7 @@
       <x:c r="K65" s="561" t="str">
         <x:f>IF(B65="","",IF(AND(B65="Phụ kiện khác",C65=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C65="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L65" s="524"/>
+      <x:c r="L65" s="627"/>
       <x:c r="M65" s="524"/>
       <x:c r="N65" s="524"/>
       <x:c r="O65" s="524"/>
@@ -4056,7 +4082,7 @@
       <x:c r="K66" s="561" t="str">
         <x:f>IF(B66="","",IF(AND(B66="Phụ kiện khác",C66=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C66="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L66" s="524"/>
+      <x:c r="L66" s="627"/>
       <x:c r="M66" s="524"/>
       <x:c r="N66" s="524"/>
       <x:c r="O66" s="524"/>
@@ -4077,7 +4103,7 @@
       <x:c r="K67" s="561" t="str">
         <x:f>IF(B67="","",IF(AND(B67="Phụ kiện khác",C67=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C67="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L67" s="524"/>
+      <x:c r="L67" s="627"/>
       <x:c r="M67" s="524"/>
       <x:c r="N67" s="524"/>
       <x:c r="O67" s="524"/>
@@ -4098,7 +4124,7 @@
       <x:c r="K68" s="561" t="str">
         <x:f>IF(B68="","",IF(AND(B68="Phụ kiện khác",C68=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C68="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L68" s="524"/>
+      <x:c r="L68" s="627"/>
       <x:c r="M68" s="524"/>
       <x:c r="N68" s="524"/>
       <x:c r="O68" s="524"/>
@@ -4119,7 +4145,7 @@
       <x:c r="K69" s="561" t="str">
         <x:f>IF(B69="","",IF(AND(B69="Phụ kiện khác",C69=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C69="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L69" s="524"/>
+      <x:c r="L69" s="627"/>
       <x:c r="M69" s="524"/>
       <x:c r="N69" s="524"/>
       <x:c r="O69" s="524"/>
@@ -4140,7 +4166,7 @@
       <x:c r="K70" s="561" t="str">
         <x:f>IF(B70="","",IF(AND(B70="Phụ kiện khác",C70=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C70="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L70" s="524"/>
+      <x:c r="L70" s="627"/>
       <x:c r="M70" s="524"/>
       <x:c r="N70" s="524"/>
       <x:c r="O70" s="524"/>
@@ -4161,7 +4187,7 @@
       <x:c r="K71" s="561" t="str">
         <x:f>IF(B71="","",IF(AND(B71="Phụ kiện khác",C71=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C71="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L71" s="524"/>
+      <x:c r="L71" s="627"/>
       <x:c r="M71" s="524"/>
       <x:c r="N71" s="524"/>
       <x:c r="O71" s="524"/>
@@ -4182,7 +4208,7 @@
       <x:c r="K72" s="561" t="str">
         <x:f>IF(B72="","",IF(AND(B72="Phụ kiện khác",C72=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C72="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L72" s="524"/>
+      <x:c r="L72" s="627"/>
       <x:c r="M72" s="524"/>
       <x:c r="N72" s="524"/>
       <x:c r="O72" s="524"/>
@@ -4203,7 +4229,7 @@
       <x:c r="K73" s="561" t="str">
         <x:f>IF(B73="","",IF(AND(B73="Phụ kiện khác",C73=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C73="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L73" s="524"/>
+      <x:c r="L73" s="627"/>
       <x:c r="M73" s="524"/>
       <x:c r="N73" s="524"/>
       <x:c r="O73" s="524"/>
@@ -4224,7 +4250,7 @@
       <x:c r="K74" s="561" t="str">
         <x:f>IF(B74="","",IF(AND(B74="Phụ kiện khác",C74=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C74="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L74" s="524"/>
+      <x:c r="L74" s="627"/>
       <x:c r="M74" s="524"/>
       <x:c r="N74" s="524"/>
       <x:c r="O74" s="524"/>
@@ -4245,7 +4271,7 @@
       <x:c r="K75" s="561" t="str">
         <x:f>IF(B75="","",IF(AND(B75="Phụ kiện khác",C75=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C75="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L75" s="524"/>
+      <x:c r="L75" s="627"/>
       <x:c r="M75" s="524"/>
       <x:c r="N75" s="524"/>
       <x:c r="O75" s="524"/>
@@ -4266,7 +4292,7 @@
       <x:c r="K76" s="561" t="str">
         <x:f>IF(B76="","",IF(AND(B76="Phụ kiện khác",C76=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C76="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L76" s="524"/>
+      <x:c r="L76" s="627"/>
       <x:c r="M76" s="524"/>
       <x:c r="N76" s="524"/>
       <x:c r="O76" s="524"/>
@@ -4287,7 +4313,7 @@
       <x:c r="K77" s="561" t="str">
         <x:f>IF(B77="","",IF(AND(B77="Phụ kiện khác",C77=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C77="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L77" s="524"/>
+      <x:c r="L77" s="627"/>
       <x:c r="M77" s="524"/>
       <x:c r="N77" s="524"/>
       <x:c r="O77" s="524"/>
@@ -4308,7 +4334,7 @@
       <x:c r="K78" s="561" t="str">
         <x:f>IF(B78="","",IF(AND(B78="Phụ kiện khác",C78=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C78="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L78" s="524"/>
+      <x:c r="L78" s="627"/>
       <x:c r="M78" s="524"/>
       <x:c r="N78" s="524"/>
       <x:c r="O78" s="524"/>
@@ -4329,7 +4355,7 @@
       <x:c r="K79" s="561" t="str">
         <x:f>IF(B79="","",IF(AND(B79="Phụ kiện khác",C79=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C79="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L79" s="524"/>
+      <x:c r="L79" s="627"/>
       <x:c r="M79" s="524"/>
       <x:c r="N79" s="524"/>
       <x:c r="O79" s="524"/>
@@ -4350,7 +4376,7 @@
       <x:c r="K80" s="561" t="str">
         <x:f>IF(B80="","",IF(AND(B80="Phụ kiện khác",C80=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C80="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L80" s="524"/>
+      <x:c r="L80" s="627"/>
       <x:c r="M80" s="524"/>
       <x:c r="N80" s="524"/>
       <x:c r="O80" s="524"/>
@@ -4371,7 +4397,7 @@
       <x:c r="K81" s="561" t="str">
         <x:f>IF(B81="","",IF(AND(B81="Phụ kiện khác",C81=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C81="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L81" s="524"/>
+      <x:c r="L81" s="627"/>
       <x:c r="M81" s="524"/>
       <x:c r="N81" s="524"/>
       <x:c r="O81" s="524"/>
@@ -4392,7 +4418,7 @@
       <x:c r="K82" s="561" t="str">
         <x:f>IF(B82="","",IF(AND(B82="Phụ kiện khác",C82=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C82="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L82" s="524"/>
+      <x:c r="L82" s="627"/>
       <x:c r="M82" s="524"/>
       <x:c r="N82" s="524"/>
       <x:c r="O82" s="524"/>
@@ -4413,7 +4439,7 @@
       <x:c r="K83" s="561" t="str">
         <x:f>IF(B83="","",IF(AND(B83="Phụ kiện khác",C83=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C83="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L83" s="524"/>
+      <x:c r="L83" s="627"/>
       <x:c r="M83" s="524"/>
       <x:c r="N83" s="524"/>
       <x:c r="O83" s="524"/>
@@ -4434,7 +4460,7 @@
       <x:c r="K84" s="561" t="str">
         <x:f>IF(B84="","",IF(AND(B84="Phụ kiện khác",C84=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C84="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L84" s="524"/>
+      <x:c r="L84" s="627"/>
       <x:c r="M84" s="524"/>
       <x:c r="N84" s="524"/>
       <x:c r="O84" s="524"/>
@@ -4455,7 +4481,7 @@
       <x:c r="K85" s="561" t="str">
         <x:f>IF(B85="","",IF(AND(B85="Phụ kiện khác",C85=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C85="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L85" s="524"/>
+      <x:c r="L85" s="627"/>
       <x:c r="M85" s="524"/>
       <x:c r="N85" s="524"/>
       <x:c r="O85" s="524"/>
@@ -4476,7 +4502,7 @@
       <x:c r="K86" s="561" t="str">
         <x:f>IF(B86="","",IF(AND(B86="Phụ kiện khác",C86=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C86="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L86" s="524"/>
+      <x:c r="L86" s="627"/>
       <x:c r="M86" s="524"/>
       <x:c r="N86" s="524"/>
       <x:c r="O86" s="524"/>
@@ -4497,7 +4523,7 @@
       <x:c r="K87" s="561" t="str">
         <x:f>IF(B87="","",IF(AND(B87="Phụ kiện khác",C87=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C87="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L87" s="524"/>
+      <x:c r="L87" s="627"/>
       <x:c r="M87" s="524"/>
       <x:c r="N87" s="524"/>
       <x:c r="O87" s="524"/>
@@ -4518,7 +4544,7 @@
       <x:c r="K88" s="561" t="str">
         <x:f>IF(B88="","",IF(AND(B88="Phụ kiện khác",C88=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C88="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L88" s="524"/>
+      <x:c r="L88" s="627"/>
       <x:c r="M88" s="524"/>
       <x:c r="N88" s="524"/>
       <x:c r="O88" s="524"/>
@@ -4539,7 +4565,7 @@
       <x:c r="K89" s="561" t="str">
         <x:f>IF(B89="","",IF(AND(B89="Phụ kiện khác",C89=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C89="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L89" s="524"/>
+      <x:c r="L89" s="627"/>
       <x:c r="M89" s="524"/>
       <x:c r="N89" s="524"/>
       <x:c r="O89" s="524"/>
@@ -4560,7 +4586,7 @@
       <x:c r="K90" s="561" t="str">
         <x:f>IF(B90="","",IF(AND(B90="Phụ kiện khác",C90=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C90="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L90" s="524"/>
+      <x:c r="L90" s="627"/>
       <x:c r="M90" s="524"/>
       <x:c r="N90" s="524"/>
       <x:c r="O90" s="524"/>
@@ -4581,7 +4607,7 @@
       <x:c r="K91" s="561" t="str">
         <x:f>IF(B91="","",IF(AND(B91="Phụ kiện khác",C91=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C91="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L91" s="524"/>
+      <x:c r="L91" s="627"/>
       <x:c r="M91" s="524"/>
       <x:c r="N91" s="524"/>
       <x:c r="O91" s="524"/>
@@ -4602,7 +4628,7 @@
       <x:c r="K92" s="561" t="str">
         <x:f>IF(B92="","",IF(AND(B92="Phụ kiện khác",C92=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C92="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L92" s="524"/>
+      <x:c r="L92" s="627"/>
       <x:c r="M92" s="524"/>
       <x:c r="N92" s="524"/>
       <x:c r="O92" s="524"/>
@@ -4623,7 +4649,7 @@
       <x:c r="K93" s="561" t="str">
         <x:f>IF(B93="","",IF(AND(B93="Phụ kiện khác",C93=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C93="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L93" s="524"/>
+      <x:c r="L93" s="627"/>
       <x:c r="M93" s="524"/>
       <x:c r="N93" s="524"/>
       <x:c r="O93" s="524"/>
@@ -4644,7 +4670,7 @@
       <x:c r="K94" s="561" t="str">
         <x:f>IF(B94="","",IF(AND(B94="Phụ kiện khác",C94=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C94="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L94" s="524"/>
+      <x:c r="L94" s="627"/>
       <x:c r="M94" s="524"/>
       <x:c r="N94" s="524"/>
       <x:c r="O94" s="524"/>
@@ -4665,7 +4691,7 @@
       <x:c r="K95" s="561" t="str">
         <x:f>IF(B95="","",IF(AND(B95="Phụ kiện khác",C95=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C95="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L95" s="524"/>
+      <x:c r="L95" s="627"/>
       <x:c r="M95" s="524"/>
       <x:c r="N95" s="524"/>
       <x:c r="O95" s="524"/>
@@ -4686,7 +4712,7 @@
       <x:c r="K96" s="561" t="str">
         <x:f>IF(B96="","",IF(AND(B96="Phụ kiện khác",C96=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C96="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L96" s="524"/>
+      <x:c r="L96" s="627"/>
       <x:c r="M96" s="524"/>
       <x:c r="N96" s="524"/>
       <x:c r="O96" s="524"/>
@@ -4707,7 +4733,7 @@
       <x:c r="K97" s="561" t="str">
         <x:f>IF(B97="","",IF(AND(B97="Phụ kiện khác",C97=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C97="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L97" s="524"/>
+      <x:c r="L97" s="627"/>
       <x:c r="M97" s="524"/>
       <x:c r="N97" s="524"/>
       <x:c r="O97" s="524"/>
@@ -4728,7 +4754,7 @@
       <x:c r="K98" s="561" t="str">
         <x:f>IF(B98="","",IF(AND(B98="Phụ kiện khác",C98=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C98="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L98" s="524"/>
+      <x:c r="L98" s="627"/>
       <x:c r="M98" s="524"/>
       <x:c r="N98" s="524"/>
       <x:c r="O98" s="524"/>
@@ -4749,7 +4775,7 @@
       <x:c r="K99" s="561" t="str">
         <x:f>IF(B99="","",IF(AND(B99="Phụ kiện khác",C99=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C99="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L99" s="524"/>
+      <x:c r="L99" s="627"/>
       <x:c r="M99" s="524"/>
       <x:c r="N99" s="524"/>
       <x:c r="O99" s="524"/>
@@ -4770,7 +4796,7 @@
       <x:c r="K100" s="561" t="str">
         <x:f>IF(B100="","",IF(AND(B100="Phụ kiện khác",C100=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C100="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L100" s="524"/>
+      <x:c r="L100" s="627"/>
       <x:c r="M100" s="524"/>
       <x:c r="N100" s="524"/>
       <x:c r="O100" s="524"/>
@@ -4791,7 +4817,7 @@
       <x:c r="K101" s="561" t="str">
         <x:f>IF(B101="","",IF(AND(B101="Phụ kiện khác",C101=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C101="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L101" s="524"/>
+      <x:c r="L101" s="627"/>
       <x:c r="M101" s="524"/>
       <x:c r="N101" s="524"/>
       <x:c r="O101" s="524"/>
@@ -4812,7 +4838,7 @@
       <x:c r="K102" s="561" t="str">
         <x:f>IF(B102="","",IF(AND(B102="Phụ kiện khác",C102=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C102="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L102" s="524"/>
+      <x:c r="L102" s="627"/>
       <x:c r="M102" s="524"/>
       <x:c r="N102" s="524"/>
       <x:c r="O102" s="524"/>
@@ -4833,7 +4859,7 @@
       <x:c r="K103" s="561" t="str">
         <x:f>IF(B103="","",IF(AND(B103="Phụ kiện khác",C103=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C103="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L103" s="524"/>
+      <x:c r="L103" s="627"/>
       <x:c r="M103" s="524"/>
       <x:c r="N103" s="524"/>
       <x:c r="O103" s="524"/>
@@ -4854,7 +4880,7 @@
       <x:c r="K104" s="561" t="str">
         <x:f>IF(B104="","",IF(AND(B104="Phụ kiện khác",C104=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C104="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L104" s="524"/>
+      <x:c r="L104" s="627"/>
       <x:c r="M104" s="524"/>
       <x:c r="N104" s="524"/>
       <x:c r="O104" s="524"/>
@@ -4875,7 +4901,7 @@
       <x:c r="K105" s="561" t="str">
         <x:f>IF(B105="","",IF(AND(B105="Phụ kiện khác",C105=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C105="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L105" s="524"/>
+      <x:c r="L105" s="627"/>
       <x:c r="M105" s="524"/>
       <x:c r="N105" s="524"/>
       <x:c r="O105" s="524"/>
@@ -4896,7 +4922,7 @@
       <x:c r="K106" s="561" t="str">
         <x:f>IF(B106="","",IF(AND(B106="Phụ kiện khác",C106=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C106="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L106" s="524"/>
+      <x:c r="L106" s="627"/>
       <x:c r="M106" s="524"/>
       <x:c r="N106" s="524"/>
       <x:c r="O106" s="524"/>
@@ -4917,7 +4943,7 @@
       <x:c r="K107" s="561" t="str">
         <x:f>IF(B107="","",IF(AND(B107="Phụ kiện khác",C107=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C107="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L107" s="524"/>
+      <x:c r="L107" s="627"/>
       <x:c r="M107" s="524"/>
       <x:c r="N107" s="524"/>
       <x:c r="O107" s="524"/>
@@ -4938,7 +4964,7 @@
       <x:c r="K108" s="561" t="str">
         <x:f>IF(B108="","",IF(AND(B108="Phụ kiện khác",C108=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C108="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L108" s="524"/>
+      <x:c r="L108" s="627"/>
       <x:c r="M108" s="524"/>
       <x:c r="N108" s="524"/>
       <x:c r="O108" s="524"/>
@@ -4959,7 +4985,7 @@
       <x:c r="K109" s="561" t="str">
         <x:f>IF(B109="","",IF(AND(B109="Phụ kiện khác",C109=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C109="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L109" s="524"/>
+      <x:c r="L109" s="627"/>
       <x:c r="M109" s="524"/>
       <x:c r="N109" s="524"/>
       <x:c r="O109" s="524"/>
@@ -4980,7 +5006,7 @@
       <x:c r="K110" s="561" t="str">
         <x:f>IF(B110="","",IF(AND(B110="Phụ kiện khác",C110=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C110="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L110" s="524"/>
+      <x:c r="L110" s="627"/>
       <x:c r="M110" s="524"/>
       <x:c r="N110" s="524"/>
       <x:c r="O110" s="524"/>
@@ -5001,7 +5027,7 @@
       <x:c r="K111" s="561" t="str">
         <x:f>IF(B111="","",IF(AND(B111="Phụ kiện khác",C111=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C111="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L111" s="524"/>
+      <x:c r="L111" s="627"/>
       <x:c r="M111" s="524"/>
       <x:c r="N111" s="524"/>
       <x:c r="O111" s="524"/>
@@ -5022,7 +5048,7 @@
       <x:c r="K112" s="561" t="str">
         <x:f>IF(B112="","",IF(AND(B112="Phụ kiện khác",C112=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C112="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L112" s="524"/>
+      <x:c r="L112" s="627"/>
       <x:c r="M112" s="524"/>
       <x:c r="N112" s="524"/>
       <x:c r="O112" s="524"/>
@@ -5043,7 +5069,7 @@
       <x:c r="K113" s="561" t="str">
         <x:f>IF(B113="","",IF(AND(B113="Phụ kiện khác",C113=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C113="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L113" s="524"/>
+      <x:c r="L113" s="627"/>
       <x:c r="M113" s="524"/>
       <x:c r="N113" s="524"/>
       <x:c r="O113" s="524"/>
@@ -5064,7 +5090,7 @@
       <x:c r="K114" s="561" t="str">
         <x:f>IF(B114="","",IF(AND(B114="Phụ kiện khác",C114=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C114="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L114" s="524"/>
+      <x:c r="L114" s="627"/>
       <x:c r="M114" s="524"/>
       <x:c r="N114" s="524"/>
       <x:c r="O114" s="524"/>
@@ -5085,7 +5111,7 @@
       <x:c r="K115" s="561" t="str">
         <x:f>IF(B115="","",IF(AND(B115="Phụ kiện khác",C115=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C115="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L115" s="524"/>
+      <x:c r="L115" s="627"/>
       <x:c r="M115" s="524"/>
       <x:c r="N115" s="524"/>
       <x:c r="O115" s="524"/>
@@ -5106,7 +5132,7 @@
       <x:c r="K116" s="561" t="str">
         <x:f>IF(B116="","",IF(AND(B116="Phụ kiện khác",C116=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C116="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L116" s="524"/>
+      <x:c r="L116" s="627"/>
       <x:c r="M116" s="524"/>
       <x:c r="N116" s="524"/>
       <x:c r="O116" s="524"/>
@@ -5127,7 +5153,7 @@
       <x:c r="K117" s="561" t="str">
         <x:f>IF(B117="","",IF(AND(B117="Phụ kiện khác",C117=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C117="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L117" s="524"/>
+      <x:c r="L117" s="627"/>
       <x:c r="M117" s="524"/>
       <x:c r="N117" s="524"/>
       <x:c r="O117" s="524"/>
@@ -5148,7 +5174,7 @@
       <x:c r="K118" s="561" t="str">
         <x:f>IF(B118="","",IF(AND(B118="Phụ kiện khác",C118=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C118="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L118" s="524"/>
+      <x:c r="L118" s="627"/>
       <x:c r="M118" s="524"/>
       <x:c r="N118" s="524"/>
       <x:c r="O118" s="524"/>
@@ -5169,7 +5195,7 @@
       <x:c r="K119" s="561" t="str">
         <x:f>IF(B119="","",IF(AND(B119="Phụ kiện khác",C119=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C119="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L119" s="524"/>
+      <x:c r="L119" s="627"/>
       <x:c r="M119" s="524"/>
       <x:c r="N119" s="524"/>
       <x:c r="O119" s="524"/>
@@ -5190,7 +5216,7 @@
       <x:c r="K120" s="561" t="str">
         <x:f>IF(B120="","",IF(AND(B120="Phụ kiện khác",C120=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C120="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L120" s="524"/>
+      <x:c r="L120" s="627"/>
       <x:c r="M120" s="524"/>
       <x:c r="N120" s="524"/>
       <x:c r="O120" s="524"/>
@@ -5211,7 +5237,7 @@
       <x:c r="K121" s="561" t="str">
         <x:f>IF(B121="","",IF(AND(B121="Phụ kiện khác",C121=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C121="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L121" s="524"/>
+      <x:c r="L121" s="627"/>
       <x:c r="M121" s="524"/>
       <x:c r="N121" s="524"/>
       <x:c r="O121" s="524"/>
@@ -5232,7 +5258,7 @@
       <x:c r="K122" s="561" t="str">
         <x:f>IF(B122="","",IF(AND(B122="Phụ kiện khác",C122=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C122="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L122" s="524"/>
+      <x:c r="L122" s="627"/>
       <x:c r="M122" s="524"/>
       <x:c r="N122" s="524"/>
       <x:c r="O122" s="524"/>
@@ -5253,7 +5279,7 @@
       <x:c r="K123" s="561" t="str">
         <x:f>IF(B123="","",IF(AND(B123="Phụ kiện khác",C123=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C123="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L123" s="524"/>
+      <x:c r="L123" s="627"/>
       <x:c r="M123" s="524"/>
       <x:c r="N123" s="524"/>
       <x:c r="O123" s="524"/>
@@ -5274,7 +5300,7 @@
       <x:c r="K124" s="561" t="str">
         <x:f>IF(B124="","",IF(AND(B124="Phụ kiện khác",C124=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C124="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L124" s="524"/>
+      <x:c r="L124" s="627"/>
       <x:c r="M124" s="524"/>
       <x:c r="N124" s="524"/>
       <x:c r="O124" s="524"/>
@@ -5295,7 +5321,7 @@
       <x:c r="K125" s="561" t="str">
         <x:f>IF(B125="","",IF(AND(B125="Phụ kiện khác",C125=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C125="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L125" s="524"/>
+      <x:c r="L125" s="627"/>
       <x:c r="M125" s="524"/>
       <x:c r="N125" s="524"/>
       <x:c r="O125" s="524"/>
@@ -5316,7 +5342,7 @@
       <x:c r="K126" s="561" t="str">
         <x:f>IF(B126="","",IF(AND(B126="Phụ kiện khác",C126=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C126="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L126" s="524"/>
+      <x:c r="L126" s="627"/>
       <x:c r="M126" s="524"/>
       <x:c r="N126" s="524"/>
       <x:c r="O126" s="524"/>
@@ -5337,7 +5363,7 @@
       <x:c r="K127" s="561" t="str">
         <x:f>IF(B127="","",IF(AND(B127="Phụ kiện khác",C127=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C127="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L127" s="524"/>
+      <x:c r="L127" s="627"/>
       <x:c r="M127" s="524"/>
       <x:c r="N127" s="524"/>
       <x:c r="O127" s="524"/>
@@ -5358,7 +5384,7 @@
       <x:c r="K128" s="561" t="str">
         <x:f>IF(B128="","",IF(AND(B128="Phụ kiện khác",C128=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C128="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L128" s="524"/>
+      <x:c r="L128" s="627"/>
       <x:c r="M128" s="524"/>
       <x:c r="N128" s="524"/>
       <x:c r="O128" s="524"/>
@@ -5379,7 +5405,7 @@
       <x:c r="K129" s="561" t="str">
         <x:f>IF(B129="","",IF(AND(B129="Phụ kiện khác",C129=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C129="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L129" s="524"/>
+      <x:c r="L129" s="627"/>
       <x:c r="M129" s="524"/>
       <x:c r="N129" s="524"/>
       <x:c r="O129" s="524"/>
@@ -5400,7 +5426,7 @@
       <x:c r="K130" s="561" t="str">
         <x:f>IF(B130="","",IF(AND(B130="Phụ kiện khác",C130=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C130="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L130" s="524"/>
+      <x:c r="L130" s="627"/>
       <x:c r="M130" s="524"/>
       <x:c r="N130" s="524"/>
       <x:c r="O130" s="524"/>
@@ -5421,7 +5447,7 @@
       <x:c r="K131" s="561" t="str">
         <x:f>IF(B131="","",IF(AND(B131="Phụ kiện khác",C131=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C131="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L131" s="524"/>
+      <x:c r="L131" s="627"/>
       <x:c r="M131" s="524"/>
       <x:c r="N131" s="524"/>
       <x:c r="O131" s="524"/>
@@ -5442,7 +5468,7 @@
       <x:c r="K132" s="561" t="str">
         <x:f>IF(B132="","",IF(AND(B132="Phụ kiện khác",C132=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C132="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L132" s="524"/>
+      <x:c r="L132" s="627"/>
       <x:c r="M132" s="524"/>
       <x:c r="N132" s="524"/>
       <x:c r="O132" s="524"/>
@@ -5463,7 +5489,7 @@
       <x:c r="K133" s="561" t="str">
         <x:f>IF(B133="","",IF(AND(B133="Phụ kiện khác",C133=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C133="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L133" s="524"/>
+      <x:c r="L133" s="627"/>
       <x:c r="M133" s="524"/>
       <x:c r="N133" s="524"/>
       <x:c r="O133" s="524"/>
@@ -5484,7 +5510,7 @@
       <x:c r="K134" s="561" t="str">
         <x:f>IF(B134="","",IF(AND(B134="Phụ kiện khác",C134=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C134="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L134" s="524"/>
+      <x:c r="L134" s="627"/>
       <x:c r="M134" s="524"/>
       <x:c r="N134" s="524"/>
       <x:c r="O134" s="524"/>
@@ -5505,7 +5531,7 @@
       <x:c r="K135" s="561" t="str">
         <x:f>IF(B135="","",IF(AND(B135="Phụ kiện khác",C135=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C135="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L135" s="524"/>
+      <x:c r="L135" s="627"/>
       <x:c r="M135" s="524"/>
       <x:c r="N135" s="524"/>
       <x:c r="O135" s="524"/>
@@ -5526,7 +5552,7 @@
       <x:c r="K136" s="561" t="str">
         <x:f>IF(B136="","",IF(AND(B136="Phụ kiện khác",C136=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C136="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L136" s="524"/>
+      <x:c r="L136" s="627"/>
       <x:c r="M136" s="524"/>
       <x:c r="N136" s="524"/>
       <x:c r="O136" s="524"/>
@@ -5547,7 +5573,7 @@
       <x:c r="K137" s="561" t="str">
         <x:f>IF(B137="","",IF(AND(B137="Phụ kiện khác",C137=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C137="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L137" s="524"/>
+      <x:c r="L137" s="627"/>
       <x:c r="M137" s="524"/>
       <x:c r="N137" s="524"/>
       <x:c r="O137" s="524"/>
@@ -5568,7 +5594,7 @@
       <x:c r="K138" s="561" t="str">
         <x:f>IF(B138="","",IF(AND(B138="Phụ kiện khác",C138=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C138="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L138" s="524"/>
+      <x:c r="L138" s="627"/>
       <x:c r="M138" s="524"/>
       <x:c r="N138" s="524"/>
       <x:c r="O138" s="524"/>
@@ -5589,7 +5615,7 @@
       <x:c r="K139" s="561" t="str">
         <x:f>IF(B139="","",IF(AND(B139="Phụ kiện khác",C139=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C139="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L139" s="524"/>
+      <x:c r="L139" s="627"/>
       <x:c r="M139" s="524"/>
       <x:c r="N139" s="524"/>
       <x:c r="O139" s="524"/>
@@ -5610,7 +5636,7 @@
       <x:c r="K140" s="561" t="str">
         <x:f>IF(B140="","",IF(AND(B140="Phụ kiện khác",C140=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C140="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L140" s="524"/>
+      <x:c r="L140" s="627"/>
       <x:c r="M140" s="524"/>
       <x:c r="N140" s="524"/>
       <x:c r="O140" s="524"/>
@@ -5631,7 +5657,7 @@
       <x:c r="K141" s="561" t="str">
         <x:f>IF(B141="","",IF(AND(B141="Phụ kiện khác",C141=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C141="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L141" s="524"/>
+      <x:c r="L141" s="627"/>
       <x:c r="M141" s="524"/>
       <x:c r="N141" s="524"/>
       <x:c r="O141" s="524"/>
@@ -5652,7 +5678,7 @@
       <x:c r="K142" s="561" t="str">
         <x:f>IF(B142="","",IF(AND(B142="Phụ kiện khác",C142=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C142="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L142" s="524"/>
+      <x:c r="L142" s="627"/>
       <x:c r="M142" s="524"/>
       <x:c r="N142" s="524"/>
       <x:c r="O142" s="524"/>
@@ -5673,7 +5699,7 @@
       <x:c r="K143" s="561" t="str">
         <x:f>IF(B143="","",IF(AND(B143="Phụ kiện khác",C143=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C143="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L143" s="524"/>
+      <x:c r="L143" s="627"/>
       <x:c r="M143" s="524"/>
       <x:c r="N143" s="524"/>
       <x:c r="O143" s="524"/>
@@ -5694,7 +5720,7 @@
       <x:c r="K144" s="561" t="str">
         <x:f>IF(B144="","",IF(AND(B144="Phụ kiện khác",C144=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C144="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L144" s="524"/>
+      <x:c r="L144" s="627"/>
       <x:c r="M144" s="524"/>
       <x:c r="N144" s="524"/>
       <x:c r="O144" s="524"/>
@@ -5715,7 +5741,7 @@
       <x:c r="K145" s="561" t="str">
         <x:f>IF(B145="","",IF(AND(B145="Phụ kiện khác",C145=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C145="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L145" s="524"/>
+      <x:c r="L145" s="627"/>
       <x:c r="M145" s="524"/>
       <x:c r="N145" s="524"/>
       <x:c r="O145" s="524"/>
@@ -5736,7 +5762,7 @@
       <x:c r="K146" s="561" t="str">
         <x:f>IF(B146="","",IF(AND(B146="Phụ kiện khác",C146=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C146="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L146" s="524"/>
+      <x:c r="L146" s="627"/>
       <x:c r="M146" s="524"/>
       <x:c r="N146" s="524"/>
       <x:c r="O146" s="524"/>
@@ -5757,7 +5783,7 @@
       <x:c r="K147" s="561" t="str">
         <x:f>IF(B147="","",IF(AND(B147="Phụ kiện khác",C147=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C147="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L147" s="524"/>
+      <x:c r="L147" s="627"/>
       <x:c r="M147" s="524"/>
       <x:c r="N147" s="524"/>
       <x:c r="O147" s="524"/>
@@ -5778,7 +5804,7 @@
       <x:c r="K148" s="561" t="str">
         <x:f>IF(B148="","",IF(AND(B148="Phụ kiện khác",C148=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C148="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L148" s="524"/>
+      <x:c r="L148" s="627"/>
       <x:c r="M148" s="524"/>
       <x:c r="N148" s="524"/>
       <x:c r="O148" s="524"/>
@@ -5799,7 +5825,7 @@
       <x:c r="K149" s="561" t="str">
         <x:f>IF(B149="","",IF(AND(B149="Phụ kiện khác",C149=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C149="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L149" s="524"/>
+      <x:c r="L149" s="627"/>
       <x:c r="M149" s="524"/>
       <x:c r="N149" s="524"/>
       <x:c r="O149" s="524"/>
@@ -5820,7 +5846,7 @@
       <x:c r="K150" s="561" t="str">
         <x:f>IF(B150="","",IF(AND(B150="Phụ kiện khác",C150=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C150="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L150" s="524"/>
+      <x:c r="L150" s="627"/>
       <x:c r="M150" s="524"/>
       <x:c r="N150" s="524"/>
       <x:c r="O150" s="524"/>
@@ -5841,7 +5867,7 @@
       <x:c r="K151" s="561" t="str">
         <x:f>IF(B151="","",IF(AND(B151="Phụ kiện khác",C151=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C151="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L151" s="524"/>
+      <x:c r="L151" s="627"/>
       <x:c r="M151" s="524"/>
       <x:c r="N151" s="524"/>
       <x:c r="O151" s="524"/>
@@ -5862,7 +5888,7 @@
       <x:c r="K152" s="561" t="str">
         <x:f>IF(B152="","",IF(AND(B152="Phụ kiện khác",C152=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C152="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L152" s="524"/>
+      <x:c r="L152" s="627"/>
       <x:c r="M152" s="524"/>
       <x:c r="N152" s="524"/>
       <x:c r="O152" s="524"/>
@@ -5883,7 +5909,7 @@
       <x:c r="K153" s="561" t="str">
         <x:f>IF(B153="","",IF(AND(B153="Phụ kiện khác",C153=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C153="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L153" s="524"/>
+      <x:c r="L153" s="627"/>
       <x:c r="M153" s="524"/>
       <x:c r="N153" s="524"/>
       <x:c r="O153" s="524"/>
@@ -5904,7 +5930,7 @@
       <x:c r="K154" s="561" t="str">
         <x:f>IF(B154="","",IF(AND(B154="Phụ kiện khác",C154=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C154="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L154" s="524"/>
+      <x:c r="L154" s="627"/>
       <x:c r="M154" s="524"/>
       <x:c r="N154" s="524"/>
       <x:c r="O154" s="524"/>
@@ -5925,7 +5951,7 @@
       <x:c r="K155" s="561" t="str">
         <x:f>IF(B155="","",IF(AND(B155="Phụ kiện khác",C155=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C155="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L155" s="524"/>
+      <x:c r="L155" s="627"/>
       <x:c r="M155" s="524"/>
       <x:c r="N155" s="524"/>
       <x:c r="O155" s="524"/>
@@ -5946,7 +5972,7 @@
       <x:c r="K156" s="561" t="str">
         <x:f>IF(B156="","",IF(AND(B156="Phụ kiện khác",C156=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C156="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L156" s="524"/>
+      <x:c r="L156" s="627"/>
       <x:c r="M156" s="524"/>
       <x:c r="N156" s="524"/>
       <x:c r="O156" s="524"/>
@@ -5967,7 +5993,7 @@
       <x:c r="K157" s="561" t="str">
         <x:f>IF(B157="","",IF(AND(B157="Phụ kiện khác",C157=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C157="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L157" s="524"/>
+      <x:c r="L157" s="627"/>
       <x:c r="M157" s="524"/>
       <x:c r="N157" s="524"/>
       <x:c r="O157" s="524"/>
@@ -5988,7 +6014,7 @@
       <x:c r="K158" s="561" t="str">
         <x:f>IF(B158="","",IF(AND(B158="Phụ kiện khác",C158=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C158="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L158" s="524"/>
+      <x:c r="L158" s="627"/>
       <x:c r="M158" s="524"/>
       <x:c r="N158" s="524"/>
       <x:c r="O158" s="524"/>
@@ -6009,7 +6035,7 @@
       <x:c r="K159" s="561" t="str">
         <x:f>IF(B159="","",IF(AND(B159="Phụ kiện khác",C159=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C159="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L159" s="524"/>
+      <x:c r="L159" s="627"/>
       <x:c r="M159" s="524"/>
       <x:c r="N159" s="524"/>
       <x:c r="O159" s="524"/>
@@ -6030,7 +6056,7 @@
       <x:c r="K160" s="561" t="str">
         <x:f>IF(B160="","",IF(AND(B160="Phụ kiện khác",C160=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C160="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L160" s="524"/>
+      <x:c r="L160" s="627"/>
       <x:c r="M160" s="524"/>
       <x:c r="N160" s="524"/>
       <x:c r="O160" s="524"/>
@@ -6051,7 +6077,7 @@
       <x:c r="K161" s="561" t="str">
         <x:f>IF(B161="","",IF(AND(B161="Phụ kiện khác",C161=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C161="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L161" s="524"/>
+      <x:c r="L161" s="627"/>
       <x:c r="M161" s="524"/>
       <x:c r="N161" s="524"/>
       <x:c r="O161" s="524"/>
@@ -6072,7 +6098,7 @@
       <x:c r="K162" s="561" t="str">
         <x:f>IF(B162="","",IF(AND(B162="Phụ kiện khác",C162=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C162="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L162" s="524"/>
+      <x:c r="L162" s="627"/>
       <x:c r="M162" s="524"/>
       <x:c r="N162" s="524"/>
       <x:c r="O162" s="524"/>
@@ -6093,7 +6119,7 @@
       <x:c r="K163" s="561" t="str">
         <x:f>IF(B163="","",IF(AND(B163="Phụ kiện khác",C163=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C163="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L163" s="524"/>
+      <x:c r="L163" s="627"/>
       <x:c r="M163" s="524"/>
       <x:c r="N163" s="524"/>
       <x:c r="O163" s="524"/>
@@ -6114,7 +6140,7 @@
       <x:c r="K164" s="561" t="str">
         <x:f>IF(B164="","",IF(AND(B164="Phụ kiện khác",C164=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C164="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L164" s="524"/>
+      <x:c r="L164" s="627"/>
       <x:c r="M164" s="524"/>
       <x:c r="N164" s="524"/>
       <x:c r="O164" s="524"/>
@@ -6135,7 +6161,7 @@
       <x:c r="K165" s="561" t="str">
         <x:f>IF(B165="","",IF(AND(B165="Phụ kiện khác",C165=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C165="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L165" s="524"/>
+      <x:c r="L165" s="627"/>
       <x:c r="M165" s="524"/>
       <x:c r="N165" s="524"/>
       <x:c r="O165" s="524"/>
@@ -6156,7 +6182,7 @@
       <x:c r="K166" s="561" t="str">
         <x:f>IF(B166="","",IF(AND(B166="Phụ kiện khác",C166=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C166="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L166" s="524"/>
+      <x:c r="L166" s="627"/>
       <x:c r="M166" s="524"/>
       <x:c r="N166" s="524"/>
       <x:c r="O166" s="524"/>
@@ -6177,7 +6203,7 @@
       <x:c r="K167" s="561" t="str">
         <x:f>IF(B167="","",IF(AND(B167="Phụ kiện khác",C167=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C167="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L167" s="524"/>
+      <x:c r="L167" s="627"/>
       <x:c r="M167" s="524"/>
       <x:c r="N167" s="524"/>
       <x:c r="O167" s="524"/>
@@ -6198,7 +6224,7 @@
       <x:c r="K168" s="561" t="str">
         <x:f>IF(B168="","",IF(AND(B168="Phụ kiện khác",C168=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C168="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L168" s="524"/>
+      <x:c r="L168" s="627"/>
       <x:c r="M168" s="524"/>
       <x:c r="N168" s="524"/>
       <x:c r="O168" s="524"/>
@@ -6219,7 +6245,7 @@
       <x:c r="K169" s="561" t="str">
         <x:f>IF(B169="","",IF(AND(B169="Phụ kiện khác",C169=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C169="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L169" s="524"/>
+      <x:c r="L169" s="627"/>
       <x:c r="M169" s="524"/>
       <x:c r="N169" s="524"/>
       <x:c r="O169" s="524"/>
@@ -6240,7 +6266,7 @@
       <x:c r="K170" s="561" t="str">
         <x:f>IF(B170="","",IF(AND(B170="Phụ kiện khác",C170=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C170="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L170" s="524"/>
+      <x:c r="L170" s="627"/>
       <x:c r="M170" s="524"/>
       <x:c r="N170" s="524"/>
       <x:c r="O170" s="524"/>
@@ -6261,7 +6287,7 @@
       <x:c r="K171" s="561" t="str">
         <x:f>IF(B171="","",IF(AND(B171="Phụ kiện khác",C171=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C171="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L171" s="524"/>
+      <x:c r="L171" s="627"/>
       <x:c r="M171" s="524"/>
       <x:c r="N171" s="524"/>
       <x:c r="O171" s="524"/>
@@ -6282,7 +6308,7 @@
       <x:c r="K172" s="561" t="str">
         <x:f>IF(B172="","",IF(AND(B172="Phụ kiện khác",C172=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C172="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L172" s="524"/>
+      <x:c r="L172" s="627"/>
       <x:c r="M172" s="524"/>
       <x:c r="N172" s="524"/>
       <x:c r="O172" s="524"/>
@@ -6303,7 +6329,7 @@
       <x:c r="K173" s="561" t="str">
         <x:f>IF(B173="","",IF(AND(B173="Phụ kiện khác",C173=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C173="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L173" s="524"/>
+      <x:c r="L173" s="627"/>
       <x:c r="M173" s="524"/>
       <x:c r="N173" s="524"/>
       <x:c r="O173" s="524"/>
@@ -6324,7 +6350,7 @@
       <x:c r="K174" s="561" t="str">
         <x:f>IF(B174="","",IF(AND(B174="Phụ kiện khác",C174=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C174="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L174" s="524"/>
+      <x:c r="L174" s="627"/>
       <x:c r="M174" s="524"/>
       <x:c r="N174" s="524"/>
       <x:c r="O174" s="524"/>
@@ -6345,7 +6371,7 @@
       <x:c r="K175" s="561" t="str">
         <x:f>IF(B175="","",IF(AND(B175="Phụ kiện khác",C175=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C175="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L175" s="524"/>
+      <x:c r="L175" s="627"/>
       <x:c r="M175" s="524"/>
       <x:c r="N175" s="524"/>
       <x:c r="O175" s="524"/>
@@ -6366,7 +6392,7 @@
       <x:c r="K176" s="561" t="str">
         <x:f>IF(B176="","",IF(AND(B176="Phụ kiện khác",C176=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C176="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L176" s="524"/>
+      <x:c r="L176" s="627"/>
       <x:c r="M176" s="524"/>
       <x:c r="N176" s="524"/>
       <x:c r="O176" s="524"/>
@@ -6387,7 +6413,7 @@
       <x:c r="K177" s="561" t="str">
         <x:f>IF(B177="","",IF(AND(B177="Phụ kiện khác",C177=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C177="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L177" s="524"/>
+      <x:c r="L177" s="627"/>
       <x:c r="M177" s="524"/>
       <x:c r="N177" s="524"/>
       <x:c r="O177" s="524"/>
@@ -6408,7 +6434,7 @@
       <x:c r="K178" s="561" t="str">
         <x:f>IF(B178="","",IF(AND(B178="Phụ kiện khác",C178=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C178="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L178" s="524"/>
+      <x:c r="L178" s="627"/>
       <x:c r="M178" s="524"/>
       <x:c r="N178" s="524"/>
       <x:c r="O178" s="524"/>
@@ -6429,7 +6455,7 @@
       <x:c r="K179" s="561" t="str">
         <x:f>IF(B179="","",IF(AND(B179="Phụ kiện khác",C179=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C179="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L179" s="524"/>
+      <x:c r="L179" s="627"/>
       <x:c r="M179" s="524"/>
       <x:c r="N179" s="524"/>
       <x:c r="O179" s="524"/>
@@ -6450,7 +6476,7 @@
       <x:c r="K180" s="561" t="str">
         <x:f>IF(B180="","",IF(AND(B180="Phụ kiện khác",C180=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C180="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L180" s="524"/>
+      <x:c r="L180" s="627"/>
       <x:c r="M180" s="524"/>
       <x:c r="N180" s="524"/>
       <x:c r="O180" s="524"/>
@@ -6471,7 +6497,7 @@
       <x:c r="K181" s="561" t="str">
         <x:f>IF(B181="","",IF(AND(B181="Phụ kiện khác",C181=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C181="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L181" s="524"/>
+      <x:c r="L181" s="627"/>
       <x:c r="M181" s="524"/>
       <x:c r="N181" s="524"/>
       <x:c r="O181" s="524"/>
@@ -6492,7 +6518,7 @@
       <x:c r="K182" s="561" t="str">
         <x:f>IF(B182="","",IF(AND(B182="Phụ kiện khác",C182=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C182="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L182" s="524"/>
+      <x:c r="L182" s="627"/>
       <x:c r="M182" s="524"/>
       <x:c r="N182" s="524"/>
       <x:c r="O182" s="524"/>
@@ -6513,7 +6539,7 @@
       <x:c r="K183" s="561" t="str">
         <x:f>IF(B183="","",IF(AND(B183="Phụ kiện khác",C183=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C183="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L183" s="524"/>
+      <x:c r="L183" s="627"/>
       <x:c r="M183" s="524"/>
       <x:c r="N183" s="524"/>
       <x:c r="O183" s="524"/>
@@ -6534,7 +6560,7 @@
       <x:c r="K184" s="561" t="str">
         <x:f>IF(B184="","",IF(AND(B184="Phụ kiện khác",C184=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C184="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L184" s="524"/>
+      <x:c r="L184" s="627"/>
       <x:c r="M184" s="524"/>
       <x:c r="N184" s="524"/>
       <x:c r="O184" s="524"/>
@@ -6555,7 +6581,7 @@
       <x:c r="K185" s="561" t="str">
         <x:f>IF(B185="","",IF(AND(B185="Phụ kiện khác",C185=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C185="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L185" s="524"/>
+      <x:c r="L185" s="627"/>
       <x:c r="M185" s="524"/>
       <x:c r="N185" s="524"/>
       <x:c r="O185" s="524"/>
@@ -6576,7 +6602,7 @@
       <x:c r="K186" s="561" t="str">
         <x:f>IF(B186="","",IF(AND(B186="Phụ kiện khác",C186=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C186="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L186" s="524"/>
+      <x:c r="L186" s="627"/>
       <x:c r="M186" s="524"/>
       <x:c r="N186" s="524"/>
       <x:c r="O186" s="524"/>
@@ -6597,7 +6623,7 @@
       <x:c r="K187" s="561" t="str">
         <x:f>IF(B187="","",IF(AND(B187="Phụ kiện khác",C187=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C187="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L187" s="524"/>
+      <x:c r="L187" s="627"/>
       <x:c r="M187" s="524"/>
       <x:c r="N187" s="524"/>
       <x:c r="O187" s="524"/>
@@ -6618,7 +6644,7 @@
       <x:c r="K188" s="561" t="str">
         <x:f>IF(B188="","",IF(AND(B188="Phụ kiện khác",C188=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C188="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L188" s="524"/>
+      <x:c r="L188" s="627"/>
       <x:c r="M188" s="524"/>
       <x:c r="N188" s="524"/>
       <x:c r="O188" s="524"/>
@@ -6639,7 +6665,7 @@
       <x:c r="K189" s="561" t="str">
         <x:f>IF(B189="","",IF(AND(B189="Phụ kiện khác",C189=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C189="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L189" s="524"/>
+      <x:c r="L189" s="627"/>
       <x:c r="M189" s="524"/>
       <x:c r="N189" s="524"/>
       <x:c r="O189" s="524"/>
@@ -6660,7 +6686,7 @@
       <x:c r="K190" s="561" t="str">
         <x:f>IF(B190="","",IF(AND(B190="Phụ kiện khác",C190=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C190="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L190" s="524"/>
+      <x:c r="L190" s="627"/>
       <x:c r="M190" s="524"/>
       <x:c r="N190" s="524"/>
       <x:c r="O190" s="524"/>
@@ -6681,7 +6707,7 @@
       <x:c r="K191" s="561" t="str">
         <x:f>IF(B191="","",IF(AND(B191="Phụ kiện khác",C191=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C191="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L191" s="524"/>
+      <x:c r="L191" s="627"/>
       <x:c r="M191" s="524"/>
       <x:c r="N191" s="524"/>
       <x:c r="O191" s="524"/>
@@ -6702,7 +6728,7 @@
       <x:c r="K192" s="561" t="str">
         <x:f>IF(B192="","",IF(AND(B192="Phụ kiện khác",C192=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C192="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L192" s="524"/>
+      <x:c r="L192" s="627"/>
       <x:c r="M192" s="524"/>
       <x:c r="N192" s="524"/>
       <x:c r="O192" s="524"/>
@@ -6723,7 +6749,7 @@
       <x:c r="K193" s="561" t="str">
         <x:f>IF(B193="","",IF(AND(B193="Phụ kiện khác",C193=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C193="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L193" s="524"/>
+      <x:c r="L193" s="627"/>
       <x:c r="M193" s="524"/>
       <x:c r="N193" s="524"/>
       <x:c r="O193" s="524"/>
@@ -6744,7 +6770,7 @@
       <x:c r="K194" s="561" t="str">
         <x:f>IF(B194="","",IF(AND(B194="Phụ kiện khác",C194=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C194="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L194" s="524"/>
+      <x:c r="L194" s="627"/>
       <x:c r="M194" s="524"/>
       <x:c r="N194" s="524"/>
       <x:c r="O194" s="524"/>
@@ -6765,7 +6791,7 @@
       <x:c r="K195" s="561" t="str">
         <x:f>IF(B195="","",IF(AND(B195="Phụ kiện khác",C195=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C195="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L195" s="524"/>
+      <x:c r="L195" s="627"/>
       <x:c r="M195" s="524"/>
       <x:c r="N195" s="524"/>
       <x:c r="O195" s="524"/>
@@ -6786,7 +6812,7 @@
       <x:c r="K196" s="561" t="str">
         <x:f>IF(B196="","",IF(AND(B196="Phụ kiện khác",C196=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C196="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L196" s="524"/>
+      <x:c r="L196" s="627"/>
       <x:c r="M196" s="524"/>
       <x:c r="N196" s="524"/>
       <x:c r="O196" s="524"/>
@@ -6807,7 +6833,7 @@
       <x:c r="K197" s="561" t="str">
         <x:f>IF(B197="","",IF(AND(B197="Phụ kiện khác",C197=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C197="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L197" s="524"/>
+      <x:c r="L197" s="627"/>
       <x:c r="M197" s="524"/>
       <x:c r="N197" s="524"/>
       <x:c r="O197" s="524"/>
@@ -6828,7 +6854,7 @@
       <x:c r="K198" s="561" t="str">
         <x:f>IF(B198="","",IF(AND(B198="Phụ kiện khác",C198=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C198="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L198" s="524"/>
+      <x:c r="L198" s="627"/>
       <x:c r="M198" s="524"/>
       <x:c r="N198" s="524"/>
       <x:c r="O198" s="524"/>
@@ -6849,7 +6875,7 @@
       <x:c r="K199" s="561" t="str">
         <x:f>IF(B199="","",IF(AND(B199="Phụ kiện khác",C199=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C199="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L199" s="524"/>
+      <x:c r="L199" s="627"/>
       <x:c r="M199" s="524"/>
       <x:c r="N199" s="524"/>
       <x:c r="O199" s="524"/>
@@ -6870,7 +6896,7 @@
       <x:c r="K200" s="561" t="str">
         <x:f>IF(B200="","",IF(AND(B200="Phụ kiện khác",C200=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C200="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L200" s="524"/>
+      <x:c r="L200" s="627"/>
       <x:c r="M200" s="524"/>
       <x:c r="N200" s="524"/>
       <x:c r="O200" s="524"/>
@@ -6891,7 +6917,7 @@
       <x:c r="K201" s="561" t="str">
         <x:f>IF(B201="","",IF(AND(B201="Phụ kiện khác",C201=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C201="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L201" s="524"/>
+      <x:c r="L201" s="627"/>
       <x:c r="M201" s="524"/>
       <x:c r="N201" s="524"/>
       <x:c r="O201" s="524"/>
@@ -6912,7 +6938,7 @@
       <x:c r="K202" s="561" t="str">
         <x:f>IF(B202="","",IF(AND(B202="Phụ kiện khác",C202=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C202="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L202" s="524"/>
+      <x:c r="L202" s="627"/>
       <x:c r="M202" s="524"/>
       <x:c r="N202" s="524"/>
       <x:c r="O202" s="524"/>
@@ -6933,7 +6959,7 @@
       <x:c r="K203" s="561" t="str">
         <x:f>IF(B203="","",IF(AND(B203="Phụ kiện khác",C203=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C203="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L203" s="524"/>
+      <x:c r="L203" s="627"/>
       <x:c r="M203" s="524"/>
       <x:c r="N203" s="524"/>
       <x:c r="O203" s="524"/>
@@ -6954,7 +6980,7 @@
       <x:c r="K204" s="561" t="str">
         <x:f>IF(B204="","",IF(AND(B204="Phụ kiện khác",C204=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C204="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L204" s="524"/>
+      <x:c r="L204" s="627"/>
       <x:c r="M204" s="524"/>
       <x:c r="N204" s="524"/>
       <x:c r="O204" s="524"/>
@@ -6975,7 +7001,7 @@
       <x:c r="K205" s="561" t="str">
         <x:f>IF(B205="","",IF(AND(B205="Phụ kiện khác",C205=""),"⚠ NHẬP TÊN PHỤ KIỆN",IF(C205="","⚠ NHẬP TÊN SẢN PHẨM","OK")))</x:f>
       </x:c>
-      <x:c r="L205" s="524"/>
+      <x:c r="L205" s="627"/>
       <x:c r="M205" s="524"/>
       <x:c r="N205" s="524"/>
       <x:c r="O205" s="524"/>
@@ -14058,7 +14084,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R785e66bddf2f4796"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree12df0ff91f420b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20186,7 +20212,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R538d624e6168480d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfeec055f2e78417f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23898,7 +23924,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc71aac9c0c804f92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d75dfd4c0414d17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23986,7 +24012,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2027d5505f9480d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ae658b729fb423f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24558,7 +24584,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra58d7c64c5b9428a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4657d96574264ba6"/>
 </x:worksheet>
 </file>
 
@@ -43897,7 +43923,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racea957e6d064456"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra707982827e14846"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -47612,7 +47638,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5885a124c3e344b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4030d06b51c84ded"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -51943,7 +51969,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b33f44b850b4482"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fd61c1471494f97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>